<commit_message>
skeleton code for all except two maps (and the word cloud is ugly as)
</commit_message>
<xml_diff>
--- a/src/data/raw/Legislature.xlsx
+++ b/src/data/raw/Legislature.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chloe\Downloads\S2 2026\FIT3179\superannuation-visualisation\superannuation\data\raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chloe\Downloads\S2 2026\FIT3179\superannuation-visualisation\superannuation\src\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6762D974-C668-4AAB-BE0A-E6700669B22A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1501FED-CA4A-4533-9B3A-DFA8B88796D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="960" yWindow="2140" windowWidth="21600" windowHeight="11180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -508,14 +508,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E36"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="40.7109375" customWidth="1"/>
+    <col min="3" max="3" width="40.7265625" customWidth="1"/>
     <col min="4" max="4" width="40" customWidth="1"/>
-    <col min="5" max="5" width="35.140625" customWidth="1"/>
+    <col min="5" max="5" width="35.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -532,7 +532,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2026</v>
       </c>
@@ -549,7 +549,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -566,7 +566,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2024</v>
       </c>
@@ -580,7 +580,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2023</v>
       </c>
@@ -594,7 +594,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2022</v>
       </c>
@@ -611,7 +611,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>2021</v>
       </c>
@@ -628,7 +628,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2020</v>
       </c>
@@ -639,7 +639,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>2019</v>
       </c>
@@ -650,7 +650,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>2018</v>
       </c>
@@ -661,7 +661,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>2017</v>
       </c>
@@ -678,7 +678,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>2016</v>
       </c>
@@ -689,7 +689,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>2015</v>
       </c>
@@ -706,7 +706,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>2014</v>
       </c>
@@ -720,7 +720,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>2013</v>
       </c>
@@ -734,7 +734,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>2012</v>
       </c>
@@ -745,7 +745,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>2011</v>
       </c>
@@ -756,7 +756,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>2010</v>
       </c>
@@ -767,7 +767,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>2009</v>
       </c>
@@ -778,7 +778,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>2008</v>
       </c>
@@ -795,7 +795,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>2007</v>
       </c>
@@ -812,7 +812,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>2006</v>
       </c>
@@ -823,7 +823,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>2005</v>
       </c>
@@ -840,7 +840,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>2004</v>
       </c>
@@ -857,7 +857,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>2003</v>
       </c>
@@ -868,7 +868,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>2002</v>
       </c>
@@ -882,7 +882,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>2001</v>
       </c>
@@ -893,7 +893,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>2000</v>
       </c>
@@ -904,7 +904,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>1999</v>
       </c>
@@ -921,7 +921,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>1998</v>
       </c>
@@ -935,7 +935,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>1997</v>
       </c>
@@ -952,7 +952,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>1996</v>
       </c>
@@ -963,7 +963,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>1995</v>
       </c>
@@ -977,7 +977,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>1994</v>
       </c>
@@ -991,7 +991,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>1993</v>
       </c>
@@ -1008,7 +1008,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>1992</v>
       </c>

</xml_diff>